<commit_message>
Leva 1: ferramentas de melhoria, causas e ações no 5W2H, prazo na meta do PDCA e ficha em dia
Revisão da tarefa 8, rodada 1.

- 5W2H, exemplo 1, "O que observar": cada causa que seguiu para o
  plano tem ação; a fila do forno ficou para o ciclo seguinte; a A5 é
  a ação de controle da causa de não detecção E1 (N35, regra N35).
- PDCA, módulo 5: a meta completa dos instrumentos ganha o prazo
  ("manter o zero por 90 dias seguidos, até 18/12/2026", I19).
- Ficha: N01 atualizada (situação calculada na figura 4 do 5W2H e
  w5_data.py alterado por P23, I19 e P22); P07 diz por que agosto
  fica em 96; N35 nova.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/5W2H/5W2H-modelo.xlsx
+++ b/5W2H/5W2H-modelo.xlsx
@@ -1954,11 +1954,11 @@
         </c:ser>
         <c:gapWidth val="120"/>
         <c:overlap val="0"/>
-        <c:axId val="34601232"/>
-        <c:axId val="20872801"/>
+        <c:axId val="52920039"/>
+        <c:axId val="82080472"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="34601232"/>
+        <c:axId val="52920039"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1990,7 +1990,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20872801"/>
+        <c:crossAx val="82080472"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1998,7 +1998,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="20872801"/>
+        <c:axId val="82080472"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2038,7 +2038,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34601232"/>
+        <c:crossAx val="52920039"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>

</xml_diff>